<commit_message>
Torrejon 9 subvencion: la firmada se llama 'anulada', va como anulada
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/docs/cruce_hojas_sf2023.xlsx
+++ b/docs/cruce_hojas_sf2023.xlsx
@@ -34,7 +34,7 @@
       <color rgb="00FFFFFF"/>
     </font>
   </fonts>
-  <fills count="6">
+  <fills count="7">
     <fill>
       <patternFill/>
     </fill>
@@ -61,6 +61,11 @@
         <fgColor rgb="00F4CCCC"/>
       </patternFill>
     </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="00D9D9D9"/>
+      </patternFill>
+    </fill>
   </fills>
   <borders count="1">
     <border>
@@ -74,7 +79,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="6">
+  <cellXfs count="7">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment vertical="center" wrapText="1"/>
@@ -89,6 +94,9 @@
       <alignment vertical="top" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="5" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="6" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment vertical="top" wrapText="1"/>
     </xf>
   </cellXfs>
@@ -4659,12 +4667,16 @@
           <t>Y2023_045</t>
         </is>
       </c>
-      <c r="B48" s="3" t="inlineStr">
-        <is>
-          <t>OK</t>
-        </is>
-      </c>
-      <c r="C48" s="2" t="inlineStr"/>
+      <c r="B48" s="6" t="inlineStr">
+        <is>
+          <t>ANULADA</t>
+        </is>
+      </c>
+      <c r="C48" s="2" t="inlineStr">
+        <is>
+          <t>RESUELTO LEYENDO: El fichero se llama 'anulada' aunque la hoja (subvención 1.500, 16-06-2023) está firmada y sellada por la comunidad: mismo criterio que 'SIN EFECTO' / 'cancelado' → anulada, se conserva.</t>
+        </is>
+      </c>
       <c r="D48" s="2" t="inlineStr">
         <is>
           <t>2023-06-16</t>

</xml_diff>